<commit_message>
Rework : Story map ajout epics
</commit_message>
<xml_diff>
--- a/docs/cadrage/story-map.xlsx
+++ b/docs/cadrage/story-map.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,19 +30,19 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="16"/>
+      <sz val="15"/>
     </font>
     <font>
       <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00E8830C"/>
-      <sz val="10"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="00444444"/>
-      <sz val="9"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -52,20 +52,8 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00222222"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <color rgb="001A1A1A"/>
       <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -98,7 +86,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="25">
     <fill>
       <patternFill/>
     </fill>
@@ -112,7 +100,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8F9FA"/>
+        <fgColor rgb="00F4F4F4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002C2C54"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000D6E6E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E6DA4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005B3FA6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000E8A8A"/>
       </patternFill>
     </fill>
     <fill>
@@ -122,12 +135,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="008B1A1A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FADADD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D6E4F0"/>
+        <fgColor rgb="00F7C5C8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008B7000"/>
       </patternFill>
     </fill>
     <fill>
@@ -137,26 +160,56 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFF0A0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A5C2A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00D4EDDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00B8E8C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003A3A3A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E2E3E5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00CCCCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00EBF4FB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00F5F0FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -165,38 +218,52 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="00BBBBBB"/>
+      <left style="medium">
+        <color rgb="00888888"/>
       </left>
-      <right style="thin">
-        <color rgb="00BBBBBB"/>
+      <right style="medium">
+        <color rgb="00888888"/>
       </right>
-      <top style="thin">
-        <color rgb="00BBBBBB"/>
+      <top style="medium">
+        <color rgb="00888888"/>
       </top>
-      <bottom style="thin">
-        <color rgb="00BBBBBB"/>
+      <bottom style="medium">
+        <color rgb="00888888"/>
       </bottom>
     </border>
     <border>
       <left style="medium">
-        <color rgb="00555555"/>
+        <color rgb="00AAAAAA"/>
       </left>
       <right style="medium">
-        <color rgb="00555555"/>
+        <color rgb="00AAAAAA"/>
       </right>
       <top style="medium">
-        <color rgb="00555555"/>
+        <color rgb="00AAAAAA"/>
       </top>
       <bottom style="medium">
-        <color rgb="00555555"/>
+        <color rgb="00AAAAAA"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -204,91 +271,122 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="17" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="20" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="22" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="22" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="23" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="23" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="22" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="24" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="24" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -656,423 +754,532 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>STORY MAP · EDUTUTOR IA — Équipe 18</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1">
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>v2.0 · post-perturbation J1 · Intégration persona enseignante (Mme Lefèvre) · Cadrage / Sprint 2 · 29/06/2026</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="16" customHeight="1">
+    <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>8 activités utilisateur × 4 niveaux MoSCoW  |  Colonnes bleutées = stories enseignant ajoutées suite à la perturbation J1</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Niveau MoSCoW</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>1. S'inscrire</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>2. Uploader un cours</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>3. Générer un quiz</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>4. Passer le quiz</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>5. Consulter résultats</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>6. Gérer compte (RGPD)</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>7. Gérer sa classe
-(Enseignant ★ J1)</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>8. Suivre ses élèves
-(Enseignant ★ J1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>MUST : MVP Release 1</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
+          <t>Epics</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Contenu pédagogique</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Apprentissage</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Compte &amp; RGPD</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Gestion classe ★ J1</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Suivi élèves ★ J1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="6" t="inlineStr"/>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>👩‍🎓 Léa</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>👩‍🏫 Mme Lefèvre</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Activités</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>S'inscrire</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Uploader un cours</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>Générer un quiz</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>Passer le quiz</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>Consulter résultats</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>Gérer son compte</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>Gérer sa classe</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>Suivre ses élèves</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="90" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>MUST
+MVP Release 1</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>US-01
-F1 — Inscription email + mot de passe
+F1 — Inscription email
++ mot de passe
 (Django Auth standard)</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C6" s="13" t="inlineStr">
         <is>
           <t>US-02
-F2 — Upload PDF ≤ 5 Mo OU saisie texte ≥ 200 car.</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
+F2 — Upload PDF ≤ 5 Mo
+OU saisie texte ≥ 200 car.</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>US-03
-F3 — Génération automatique de 10 QCM
-via Llama 3.1 8B (Ollama local)</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
+F3 — Génération auto
+de 10 QCM via
+Llama 3.1 8B (Ollama)</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
         <is>
           <t>US-04
-F4 — Soumission + correction automatique
-(1 bonne réponse / QCM)</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
+F4 — Soumission +
+correction automatique
+(1 bonne réponse/QCM)</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>US-05
-F5 — Score /10 + détail bonnes/mauvaises réponses</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
+F5 — Score /10 +
+détail bonnes/
+mauvaises réponses</t>
+        </is>
+      </c>
+      <c r="G6" s="13" t="inlineStr">
         <is>
           <t>US-06
-F6 — Historique persistant des quizz par utilisateur</t>
-        </is>
-      </c>
-      <c r="H5" s="8" t="inlineStr">
+F6 — Historique
+persistant des quizz
+par utilisateur</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>US-07
-F7 — Création de classe avec code unique
-(1 code par groupe, transmis aux élèves)</t>
-        </is>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
+F7 — Création de classe
+avec code unique
+(1 code par groupe)</t>
+        </is>
+      </c>
+      <c r="I6" s="14" t="inlineStr">
         <is>
           <t>US-08
-F8 — Tableau de bord progression élèves
-(scores, dernière activité par étudiant)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>SHOULD : Release 2</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
+F8 — Dashboard
+progression élèves
+(scores + activité)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="90" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>SHOULD
+Release 2</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>US-09
-Reset password par email
+Reset password
+par email
 (lien magique 24 h)</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
         <is>
           <t>US-10
-Multi-cours : bibliothèque personnelle
-de cours uploadés</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
+Multi-cours :
+bibliothèque
+personnelle</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
         <is>
           <t>US-11
-Choix du niveau de difficulté
-+ nombre de questions (5-20)</t>
-        </is>
-      </c>
-      <c r="E6" s="10" t="inlineStr">
+Choix du niveau
+de difficulté +
+nombre questions (5-20)</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
         <is>
           <t>US-12
-Mode timer optionnel par question
+Mode timer
+optionnel par question
 (10-30 s configurable)</t>
         </is>
       </c>
-      <c r="F6" s="10" t="inlineStr">
+      <c r="F7" s="16" t="inlineStr">
         <is>
           <t>US-13
-Dashboard progression par chapitre / cours</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
+Dashboard
+progression par
+chapitre / cours</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
         <is>
           <t>US-14
-Export RGPD complet (JSON + CSV,
+Export RGPD complet
+(JSON + CSV,
 Art. 15 / 20)</t>
         </is>
       </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="H7" s="17" t="inlineStr">
         <is>
           <t>US-15
-Fil de questions élève → prof intégré
-(réponse depuis l'app)</t>
-        </is>
-      </c>
-      <c r="I6" s="8" t="inlineStr">
+Fil questions
+élève → prof intégré
+(réponse depuis app)</t>
+        </is>
+      </c>
+      <c r="I7" s="17" t="inlineStr">
         <is>
           <t>US-16
-Alerte décrochage automatique
-(élève inactif &gt; 7 j ou score &lt; 40 %)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="80" customHeight="1">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>COULD : Release 2</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
+Alerte décrochage
+auto (inactif &gt; 7 j
+ou score &lt; 40 %)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="90" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>COULD
+Release 2</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
         <is>
           <t>US-17
-Login social Google / Apple OAuth</t>
-        </is>
-      </c>
-      <c r="C7" s="12" t="inlineStr">
+Login social
+Google / Apple OAuth</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
         <is>
           <t>US-18
-Import d'un cours depuis une URL
+Import cours
+depuis une URL
 (article web, blog)</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
+      <c r="D8" s="19" t="inlineStr">
         <is>
           <t>US-19
-Mode questions ouvertes
-(correction LLM avec barème)</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
+Mode questions
+ouvertes (correction
+LLM avec barème)</t>
+        </is>
+      </c>
+      <c r="E8" s="19" t="inlineStr">
         <is>
           <t>US-20
-Mode flashcards type Anki
+Mode flashcards
+type Anki
 (révision espacée)</t>
         </is>
       </c>
-      <c r="F7" s="12" t="inlineStr">
+      <c r="F8" s="19" t="inlineStr">
         <is>
           <t>US-21
-Identification automatique des lacunes
+Identification auto
+des lacunes
 par chapitre</t>
         </is>
       </c>
-      <c r="G7" s="12" t="inlineStr">
+      <c r="G8" s="19" t="inlineStr">
         <is>
           <t>US-22
-Suppression compte + données
-(RGPD Art. 17, droit à l'oubli)</t>
-        </is>
-      </c>
-      <c r="H7" s="8" t="inlineStr">
+Suppression compte
++ données
+(RGPD Art. 17)</t>
+        </is>
+      </c>
+      <c r="H8" s="20" t="inlineStr">
         <is>
           <t>US-23
-Mode preview quiz avant publication
-(enseignant valide les QCM)</t>
-        </is>
-      </c>
-      <c r="I7" s="8" t="inlineStr">
+Mode preview quiz
+avant publication
+(enseignant valide)</t>
+        </is>
+      </c>
+      <c r="I8" s="20" t="inlineStr">
         <is>
           <t>US-24
-Envoi de conseils ciblés aux élèves
-depuis le dashboard enseignant</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="80" customHeight="1">
-      <c r="A8" s="13" t="inlineStr">
-        <is>
-          <t>WON'T (this time)</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="inlineStr">
+Envoi conseils
+ciblés aux élèves
+depuis dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="90" customHeight="1">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>WON'T
+(this time)</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
         <is>
           <t>US-25
-SSO entreprise SAML / OIDC
+SSO entreprise
+SAML / OIDC
 (B2B Release 3+)</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="C9" s="22" t="inlineStr">
         <is>
           <t>US-26
-Source vidéo ou audio
-(transcription Whisper — coûteuse)</t>
-        </is>
-      </c>
-      <c r="D8" s="14" t="inlineStr">
+Source vidéo/audio
+(transcription
+Whisper — coûteuse)</t>
+        </is>
+      </c>
+      <c r="D9" s="22" t="inlineStr">
         <is>
           <t>US-27
-Compétition multi-joueurs
+Compétition
+multi-joueurs
 (hors cible primaire)</t>
         </is>
       </c>
-      <c r="E8" s="14" t="inlineStr">
+      <c r="E9" s="22" t="inlineStr">
         <is>
           <t>US-28
-Mode IA conversationnelle
-(chatbot type Khanmigo)</t>
-        </is>
-      </c>
-      <c r="F8" s="14" t="inlineStr">
+Mode IA
+conversationnelle
+(chatbot Khanmigo)</t>
+        </is>
+      </c>
+      <c r="F9" s="22" t="inlineStr">
         <is>
           <t>US-29
-Stats temps réel collectives
-(besoin marginal MVP)</t>
-        </is>
-      </c>
-      <c r="G8" s="14" t="inlineStr">
+Stats temps réel
+collectives
+(besoin marginal)</t>
+        </is>
+      </c>
+      <c r="G9" s="22" t="inlineStr">
         <is>
           <t>US-30
-Personnalisation thème UI
-(thème sombre déjà imposé)</t>
-        </is>
-      </c>
-      <c r="H8" s="8" t="inlineStr">
+Personnalisation
+thème UI
+(thème sombre imposé)</t>
+        </is>
+      </c>
+      <c r="H9" s="23" t="inlineStr">
         <is>
           <t>US-31
-Édition manuelle d'une question générée
-→ Release 3 (complexité UX)</t>
-        </is>
-      </c>
-      <c r="I8" s="8" t="inlineStr">
+Édition manuelle
+d'une question
+→ Release 3</t>
+        </is>
+      </c>
+      <c r="I9" s="23" t="inlineStr">
         <is>
           <t>US-32
-Dashboard ROI exportable pour direction
-→ Release 3 (B2B scope)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="15" t="inlineStr">
+Dashboard ROI
+exportable direction
+→ Release 3 (B2B)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="24" t="inlineStr">
         <is>
           <t>LÉGENDE</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="16" t="inlineStr">
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="25" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="B11" s="17" t="inlineStr">
+      <c r="B12" s="26" t="inlineStr">
         <is>
           <t>Sans cette story, le produit n'a pas de sens. Engagement Sprint 1-5.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="27" t="inlineStr">
         <is>
           <t>SHOULD</t>
         </is>
       </c>
-      <c r="B12" s="19" t="inlineStr">
+      <c r="B13" s="28" t="inlineStr">
         <is>
           <t>Important, à inclure si capacité disponible. Engagement Sprint 6-7.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="20" t="inlineStr">
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>COULD</t>
         </is>
       </c>
-      <c r="B13" s="21" t="inlineStr">
+      <c r="B14" s="30" t="inlineStr">
         <is>
           <t>Bonus apprécié si temps en surplus. Sprint 7 si la R1 a été vite.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="22" t="inlineStr">
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="31" t="inlineStr">
         <is>
           <t>WON'T</t>
         </is>
       </c>
-      <c r="B14" s="23" t="inlineStr">
+      <c r="B15" s="32" t="inlineStr">
         <is>
           <t>Décision EXPLICITE de ne pas faire cette release. À documenter.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="24" t="inlineStr">
-        <is>
-          <t>★ Enseignant (J1)</t>
-        </is>
-      </c>
-      <c r="B15" s="25" t="inlineStr">
-        <is>
-          <t>Stories ajoutées post-perturbation J1 — persona Mme Lefèvre intégrée au scope (Customer Journey v2.0). Colonnes 7 &amp; 8 dédiées.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="52" customHeight="1">
-      <c r="A17" s="26" t="inlineStr">
-        <is>
-          <t>★ PERTURBATION J1 — Le périmètre produit a été élargi pour inclure le persona enseignant (Mme Lefèvre, Customer Journey v2.0). Deux nouvelles activités utilisateur ont été ajoutées : «Gérer sa classe» (col. 7) et «Suivre ses élèves» (col. 8). Les stories enseignant MUST (US-07, US-08) sont intégrées dans le MVP Release 1. Les autres stories enseignant suivent la priorisation MoSCoW standard.</t>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="33" t="inlineStr">
+        <is>
+          <t>★ Perturbation J1</t>
+        </is>
+      </c>
+      <c r="B16" s="34" t="inlineStr">
+        <is>
+          <t>Colonnes 7 &amp; 8 ajoutées suite à la perturbation J1 — persona Mme Lefèvre (Customer Journey v2.0).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="35" t="inlineStr">
+        <is>
+          <t>👩‍🎓 Léa</t>
+        </is>
+      </c>
+      <c r="B17" s="36" t="inlineStr">
+        <is>
+          <t>Persona étudiante (cible primaire) — parcours Découverte → Recommandation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="33" t="inlineStr">
+        <is>
+          <t>👩‍🏫 Mme Lefèvre</t>
+        </is>
+      </c>
+      <c r="B18" s="34" t="inlineStr">
+        <is>
+          <t>Persona enseignante (ajoutée J1) — parcours Découverte → Recommandation direction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="42" customHeight="1">
+      <c r="A20" s="37" t="inlineStr">
+        <is>
+          <t>★ PERTURBATION J1 — Périmètre élargi pour inclure le persona enseignant (Mme Lefèvre). 2 nouveaux Epics : «Gestion classe» + «Suivi élèves». 8 nouvelles US (US-07/08 MUST · US-15/16 SHOULD · US-23/24 COULD · US-31/32 WON'T). Aligné avec Customer Journey v2.0.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="15">
     <mergeCell ref="B12:I12"/>
     <mergeCell ref="B13:I13"/>
+    <mergeCell ref="B18:I18"/>
     <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A11:I11"/>
     <mergeCell ref="B15:I15"/>
-    <mergeCell ref="A10:I10"/>
-    <mergeCell ref="B11:I11"/>
+    <mergeCell ref="B16:I16"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="B4:G4"/>
     <mergeCell ref="B14:I14"/>
-    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="A20:I20"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="B17:I17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1084,7 +1291,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1092,93 +1299,105 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="27" t="inlineStr">
+      <c r="A1" s="38" t="inlineStr">
         <is>
           <t>IDENTIFICATION DU DOCUMENT — Story Map EduTutor IA</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="28" t="inlineStr">
+      <c r="A2" s="39" t="inlineStr">
         <is>
           <t>Équipe n°</t>
         </is>
       </c>
-      <c r="B2" s="29" t="inlineStr">
+      <c r="B2" s="40" t="inlineStr">
         <is>
           <t>18</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="30" t="inlineStr">
+      <c r="A3" s="41" t="inlineStr">
         <is>
           <t>Membres</t>
         </is>
       </c>
-      <c r="B3" s="31" t="inlineStr">
+      <c r="B3" s="42" t="inlineStr">
         <is>
           <t>Evan MARTIN, Maxime DANINO, Meddy GARCIA, Quentin CHASTEL, Mell CANAC</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="28" t="inlineStr">
+      <c r="A4" s="39" t="inlineStr">
         <is>
           <t>Sprint concerné</t>
         </is>
       </c>
-      <c r="B4" s="29" t="inlineStr">
-        <is>
-          <t>Cadrage / Sprint 2 - post-perturbation J1 Produit / Scope</t>
+      <c r="B4" s="40" t="inlineStr">
+        <is>
+          <t>Cadrage / Sprint 2 — post-perturbation J1 Produit / Scope</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="30" t="inlineStr">
+      <c r="A5" s="41" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="B5" s="31" t="inlineStr">
-        <is>
-          <t>v2.0 (post-perturbation J1 - intégration persona enseignante)</t>
+      <c r="B5" s="42" t="inlineStr">
+        <is>
+          <t>v2.0 (post-perturbation J1 — intégration persona enseignante)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="28" t="inlineStr">
+      <c r="A6" s="39" t="inlineStr">
         <is>
           <t>Date de remise</t>
         </is>
       </c>
-      <c r="B6" s="29" t="inlineStr">
+      <c r="B6" s="40" t="inlineStr">
         <is>
           <t>29/06/2026 16h00</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="30" t="inlineStr">
+      <c r="A7" s="41" t="inlineStr">
         <is>
           <t>Statut</t>
         </is>
       </c>
-      <c r="B7" s="31" t="inlineStr">
+      <c r="B7" s="42" t="inlineStr">
         <is>
           <t>En revue PO</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="28" t="inlineStr">
-        <is>
-          <t>Contexte perturbation</t>
-        </is>
-      </c>
-      <c r="B8" s="29" t="inlineStr">
-        <is>
-          <t>Suite à la perturbation J1, le périmètre produit a été élargi pour intégrer le persona enseignant (Mme Lefèvre). La Customer Journey v2.0 introduit 2 nouveaux parcours (enseignant + établissement). La Story Map v2.0 ajoute en conséquence 2 nouvelles colonnes activités : «Gérer sa classe» et «Suivre ses élèves», avec 8 nouvelles user stories (US-07 à US-08 en MUST, US-15/16 en SHOULD, US-23/24 en COULD, US-31/32 en WON'T).</t>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="39" t="inlineStr">
+        <is>
+          <t>Personas couverts</t>
+        </is>
+      </c>
+      <c r="B8" s="40" t="inlineStr">
+        <is>
+          <t>👩‍🎓 Léa Martin (étudiante, cible primaire) · 👩‍🏫 Mme Lefèvre (enseignante, ajoutée J1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="44" customHeight="1">
+      <c r="A9" s="41" t="inlineStr">
+        <is>
+          <t>Perturbation J1</t>
+        </is>
+      </c>
+      <c r="B9" s="42" t="inlineStr">
+        <is>
+          <t>Le périmètre produit a été élargi pour intégrer le persona enseignant (Mme Lefèvre). La Customer Journey v2.0 documente 3 parcours (étudiant, enseignant, établissement). La Story Map v2.0 ajoute 2 Epics (colonnes H &amp; I) et 8 nouvelles user stories (US-07 à US-08 MUST · US-15/16 SHOULD · US-23/24 COULD · US-31/32 WON'T).</t>
         </is>
       </c>
     </row>

</xml_diff>